<commit_message>
Testing import = export & edited README.md
</commit_message>
<xml_diff>
--- a/client-course-schedulizer/csv/Schedulizer_Course_Sections_Test.xlsx
+++ b/client-course-schedulizer/csv/Schedulizer_Course_Sections_Test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10119"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\minji\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eunhyukdoo/Desktop/Senior Project/course-schedulizer/client-course-schedulizer/csv/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3505CC55-9E87-4B5C-998F-0142F3AC83B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E666D7A-C9DF-F94E-90D3-DC1EC44FACD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4120" yWindow="2140" windowWidth="23260" windowHeight="13180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Schedulizer Course Sections" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="53">
   <si>
     <t>Department</t>
   </si>
@@ -189,6 +189,18 @@
   <si>
     <t>SB 372
 SC 120</t>
+  </si>
+  <si>
+    <t>Derek Schuurman</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>NH 100</t>
+  </si>
+  <si>
+    <t>Perspectives on Computing</t>
   </si>
 </sst>
 </file>
@@ -199,7 +211,7 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -223,7 +235,7 @@
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -237,7 +249,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -260,17 +272,63 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1" readingOrder="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -645,33 +703,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="36.296875" customWidth="1"/>
-    <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="3" width="7.09765625" customWidth="1"/>
-    <col min="4" max="4" width="7.69921875" customWidth="1"/>
-    <col min="5" max="5" width="7.59765625" customWidth="1"/>
-    <col min="6" max="6" width="5.59765625" customWidth="1"/>
-    <col min="7" max="7" width="8.69921875" customWidth="1"/>
-    <col min="8" max="8" width="41.69921875" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="8.8984375" customWidth="1"/>
-    <col min="11" max="11" width="9.3984375" customWidth="1"/>
-    <col min="12" max="12" width="9.69921875" customWidth="1"/>
-    <col min="13" max="13" width="13.69921875" customWidth="1"/>
-    <col min="14" max="14" width="10.09765625" customWidth="1"/>
-    <col min="15" max="15" width="13.69921875" customWidth="1"/>
-    <col min="16" max="16" width="37.296875" customWidth="1"/>
-    <col min="17" max="17" width="16.296875" customWidth="1"/>
-    <col min="18" max="18" width="7.09765625" customWidth="1"/>
-    <col min="19" max="19" width="20.09765625" customWidth="1"/>
-    <col min="20" max="20" width="23.296875" customWidth="1"/>
-    <col min="21" max="21" width="7.8984375" customWidth="1"/>
-    <col min="22" max="22" width="7.296875" customWidth="1"/>
+    <col min="1" max="1" width="14.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="33.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="6.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16" style="2" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="23.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" ht="23.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -739,205 +798,266 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:22" ht="30" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:22" ht="30" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="3">
         <v>1</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="3">
         <v>1</v>
       </c>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2" t="s">
+      <c r="K2" s="3"/>
+      <c r="L2" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="O2" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="P2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="Q2" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="R2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="S2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="T2" s="2" t="s">
+      <c r="T2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="U2" s="2">
+      <c r="U2" s="3">
         <v>23</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="3">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="30" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:22" ht="30" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="3">
         <v>4</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="3">
         <v>4</v>
       </c>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2" t="s">
+      <c r="K3" s="3"/>
+      <c r="L3" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="M3" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N3" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="O3" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="P3" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="Q3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="R3" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="S3" s="2" t="s">
+      <c r="S3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="T3" s="2" t="s">
+      <c r="T3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="U3" s="2">
+      <c r="U3" s="3">
         <v>37</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="3">
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:22" ht="75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:22" ht="75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="4">
         <v>4</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="4">
         <v>4</v>
       </c>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2" t="s">
+      <c r="K4" s="4"/>
+      <c r="L4" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="M4" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="N4" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="O4" s="2" t="s">
+      <c r="O4" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="P4" s="2" t="s">
+      <c r="P4" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="Q4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="R4" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="S4" s="2" t="s">
+      <c r="S4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="T4" s="2" t="s">
+      <c r="T4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="U4" s="2">
+      <c r="U4" s="4">
         <v>27</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="4">
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:22" ht="46.8" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:22" ht="46.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="6">
+        <v>384</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I5" s="6">
+        <v>4</v>
+      </c>
+      <c r="J5" s="6">
+        <v>4</v>
+      </c>
+      <c r="K5" s="6"/>
+      <c r="L5" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="N5" s="6">
+        <v>100</v>
+      </c>
+      <c r="O5" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q5" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="R5" s="8">
+        <v>300</v>
+      </c>
+      <c r="S5" s="6"/>
+      <c r="T5" s="6"/>
+      <c r="U5" s="6">
+        <v>24</v>
+      </c>
+      <c r="V5" s="6">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="1" right="1" top="1" bottom="1" header="1" footer="1"/>
@@ -947,15 +1067,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E0E33639CAF97B4BA8FEDFADD23E9349" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f741c46407df61763e17643779e0dcbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cd7edf1e-52c5-42e9-9a2d-c903a57287a0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6f4b092aa2accef1d678c45dc91bcd1e" ns2:_="">
     <xsd:import namespace="cd7edf1e-52c5-42e9-9a2d-c903a57287a0"/>
@@ -1125,6 +1236,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -1132,14 +1252,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F89678A-374C-4DCA-9A34-BE92956AEC1C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F4E9A26D-603C-488F-8E2B-7F65D132BAE6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1157,6 +1269,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F89678A-374C-4DCA-9A34-BE92956AEC1C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C8EBAC1-2D17-41E0-A8D5-16EBC6461C07}">
   <ds:schemaRefs>

</xml_diff>